<commit_message>
Add Apex Clearing broker, universal left-shift QC, Robinhood test case
- New broker: Apex Clearing (alternating desc/data rows, YYYY-MM-DD dates,
  multi-sheet with description carry-across, 11 txns verified)
- pdf_qc.py Pass 2: universal left-shift / empty-cell-collapse fix
  (Date Acquired + Gain/Loss repositioning), gain_loss_col_idx and
  fed_tax_col_idx added to all BROKER_CONFIG entries
- drake_mapper.py: YYYY-MM-DD date format support, Apex column mapping
- Robinhood added to regression suite (48 txns)
- Test data reorganized: renamed inputs in passedtestcases, cleaned up
  testdata/ (old scratch files removed, pending Schwab files remain)
- 7/7 regression tests green

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testdata/passedtestcases/fidelity_drake_import am12025.xlsx
+++ b/testdata/passedtestcases/fidelity_drake_import am12025.xlsx
@@ -1,26 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UN\fractals\VibeCoding\ClaudeCode\testdata\passedtestcases\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7CC93A-720B-4815-BA32-11A1112B5FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Drake_Import" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>TSJ</t>
   </si>
@@ -67,28 +61,31 @@
     <t>Wash Sale Loss</t>
   </si>
   <si>
+    <t>Fed Tax Withheld</t>
+  </si>
+  <si>
     <t>RHEINMETALL AG UNSP ADR EACH REPR 0.2 OR, RNMBY, 76206K107</t>
   </si>
   <si>
+    <t>UNITED STATES TREAS SER AC-2025 0.25000%, 91282CAJ0</t>
+  </si>
+  <si>
+    <t>WESTERN ALLIANCE BANCORP, WAL, 957638109</t>
+  </si>
+  <si>
     <t>03/18/2025</t>
   </si>
   <si>
+    <t>12/31/2024</t>
+  </si>
+  <si>
+    <t>01/28/2025</t>
+  </si>
+  <si>
     <t>05/02/2025</t>
   </si>
   <si>
-    <t>UNITED STATES TREAS SER AC-2025 0.25000%, 91282CAJ0</t>
-  </si>
-  <si>
-    <t>12/31/2024</t>
-  </si>
-  <si>
     <t>09/02/2025</t>
-  </si>
-  <si>
-    <t>WESTERN ALLIANCE BANCORP, WAL, 957638109</t>
-  </si>
-  <si>
-    <t>01/28/2025</t>
   </si>
   <si>
     <t>02/18/2025</t>
@@ -97,11 +94,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-  </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,7 +106,10 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -150,26 +147,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -457,27 +445,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="3.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="60.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -523,110 +495,99 @@
       <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16">
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2">
+        <v>1072.02</v>
+      </c>
+      <c r="L2">
+        <v>934.01</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="2">
-        <v>1072.02</v>
-      </c>
-      <c r="L2" s="2">
-        <v>934.01</v>
-      </c>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
+      <c r="G3" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3">
+        <v>12000</v>
+      </c>
+      <c r="L3">
+        <v>11692.56</v>
+      </c>
+      <c r="N3">
+        <v>307.44</v>
+      </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F3" t="s">
+    <row r="4" spans="1:16">
+      <c r="F4" t="s">
         <v>18</v>
       </c>
-      <c r="G3" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" t="s">
-        <v>20</v>
-      </c>
-      <c r="K3" s="2">
-        <v>12000</v>
-      </c>
-      <c r="L3" s="2">
-        <v>11692.56</v>
-      </c>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2">
-        <v>307.44</v>
-      </c>
-      <c r="O3" s="2"/>
+      <c r="G4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4">
+        <v>51.45</v>
+      </c>
+      <c r="L4">
+        <v>50.59</v>
+      </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F4" t="s">
+    <row r="5" spans="1:16">
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
         <v>21</v>
       </c>
-      <c r="G4" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" s="2">
-        <v>51.45</v>
-      </c>
-      <c r="L4" s="2">
-        <v>50.59</v>
-      </c>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
+      <c r="H5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5">
+        <v>1122.06</v>
+      </c>
+      <c r="L5">
+        <v>1098.94</v>
+      </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F5" t="s">
+    <row r="6" spans="1:16">
+      <c r="F6" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" t="s">
         <v>21</v>
       </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" t="s">
-        <v>23</v>
-      </c>
-      <c r="K5" s="2">
-        <v>1122.06</v>
-      </c>
-      <c r="L5" s="2">
-        <v>1098.94</v>
-      </c>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" t="s">
-        <v>22</v>
-      </c>
       <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="K6" s="2">
+        <v>24</v>
+      </c>
+      <c r="K6">
         <v>51.47</v>
       </c>
-      <c r="L6" s="2">
+      <c r="L6">
         <v>50.39</v>
       </c>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>